<commit_message>
feat:agregar action para exportar anuncios
</commit_message>
<xml_diff>
--- a/app/Filament/Clusters/Sil/Resources/Anuncios/Template/template_exportar_anuncios.xlsx
+++ b/app/Filament/Clusters/Sil/Resources/Anuncios/Template/template_exportar_anuncios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dacuna\Herd\itse-app\app\Filament\Clusters\Sil\Resources\Anuncios\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3FDC017-8935-4DA2-B032-55B7E9E6B105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1F14342-9EF8-4216-A2C8-9A57D868586B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3480" yWindow="4380" windowWidth="21600" windowHeight="11295" xr2:uid="{38051A38-48E2-4EA3-9221-DFEB0C6515DE}"/>
+    <workbookView xWindow="3480" yWindow="4290" windowWidth="21600" windowHeight="11295" xr2:uid="{38051A38-48E2-4EA3-9221-DFEB0C6515DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>